<commit_message>
feat(erp): read-only Ecount comparison (964 items) and Naver probe tools
</commit_message>
<xml_diff>
--- a/reports/data/procurement/bid_analysis.xlsx
+++ b/reports/data/procurement/bid_analysis.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,21 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,278 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>bid_no</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>agency</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>estimated_price</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>bid_amount</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>winning_bid</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>bid_rate_pct</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>bidders</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>close_date</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>detail_url</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>cgi_categories</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>cgi_relevant</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>data_source</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>R26BK00000001-000</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>샘플 IT 용역 공고 A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>샘플 발주기관</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>용역</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>100000000</v>
-      </c>
-      <c r="H2" t="n">
-        <v>89500000</v>
-      </c>
-      <c r="I2" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>낙찰</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-g2b\data\procurement\sample_bids.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>R26BK00000002-000</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>샘플 IT 용역 공고 B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>샘플 발주기관</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>용역</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>50000000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>47200000</v>
-      </c>
-      <c r="I3" t="n">
-        <v>94.40000000000001</v>
-      </c>
-      <c r="J3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>낙찰</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-g2b\data\procurement\sample_bids.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>R26BK00000003-000</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>샘플 물품 공고 C</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>샘플 발주기관</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>물품</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>유찰</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-g2b\data\procurement\sample_bids.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>R26BK00000004-000</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>샘플 공사 공고 D</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>샘플 발주기관</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>공사</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>200000000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>178000000</v>
-      </c>
-      <c r="I5" t="n">
-        <v>89</v>
-      </c>
-      <c r="J5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>낙찰</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-g2b\data\procurement\sample_bids.json</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve procurement report conflicts
</commit_message>
<xml_diff>
--- a/reports/data/procurement/bid_analysis.xlsx
+++ b/reports/data/procurement/bid_analysis.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +422,278 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>bid_no</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>agency</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>estimated_price</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>bid_amount</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>winning_bid</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>bid_rate_pct</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>bidders</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>close_date</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>detail_url</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>cgi_categories</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>cgi_relevant</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>data_source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R26BK00000001-000</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>샘플 IT 용역 공고 A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>샘플 발주기관</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>용역</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>89500000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>낙찰</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R26BK00000002-000</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>샘플 IT 용역 공고 B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>샘플 발주기관</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>용역</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="H3" t="n">
+        <v>47200000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>낙찰</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R26BK00000003-000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>샘플 물품 공고 C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>샘플 발주기관</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>물품</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>유찰</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R26BK00000004-000</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>샘플 공사 공고 D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>샘플 발주기관</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>공사</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>178000000</v>
+      </c>
+      <c r="I5" t="n">
+        <v>89</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>낙찰</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(procurement): recover G2B collection from derailed mall debug, add robust Playwright notice collector
- Root cause: debug7.js waited on window.CGI_PRODUCTS from CGI mall staff.html
  (site/data/products.js), not 나라장터; LOCAL2 storefront/quote code left untouched.
- Add tools/procurement/g2b_notice_collector.js: staged load logging, HTTP status,
  final URL, JS-error capture, DOM+network extraction of real notice rows, bounded
  waits (no fixed-global), reuse of open browser (--cdp/--ws/--profile), minimal
  failure diagnostics. Output feeds g2b_bid_analysis normalize/dedupe/export.
- Preserve notice_date (공고일) through the Python normalizer.
- Selftest validates extraction against a portal-shaped fixture; live run against
  g2b.go.kr reports genuine 0 (OIDC SSO + WebSquare browser-gating), no fabrication.
</commit_message>
<xml_diff>
--- a/reports/data/procurement/bid_analysis.xlsx
+++ b/reports/data/procurement/bid_analysis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,20 +488,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>notice_date</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>detail_url</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>cgi_categories</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>cgi_relevant</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
@@ -510,65 +515,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>R26BK00000001-000</t>
+          <t>CGI-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>샘플 IT 용역 공고 A</t>
+          <t>공공기관 음향장비 납품 및 설치</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>샘플 발주기관</t>
+          <t>샘플 공공기관</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>서울</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>용역</t>
+          <t>물품</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>100000000</v>
+        <v>120000000</v>
       </c>
       <c r="H2" t="n">
-        <v>89500000</v>
+        <v>108000000</v>
       </c>
       <c r="I2" t="n">
-        <v>89.5</v>
+        <v>90</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>낙찰</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>20260901</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>음향장비;공공방송설비;기자재납품</t>
+        </is>
+      </c>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>file:data/procurement/sample_cgi_bids.json</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R26BK00000002-000</t>
+          <t>CGI-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>샘플 IT 용역 공고 B</t>
+          <t>학교 방송설비 유지보수 용역</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>샘플 발주기관</t>
+          <t>샘플 교육청</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>경기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -577,13 +601,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>50000000</v>
+        <v>45000000</v>
       </c>
       <c r="H3" t="n">
-        <v>47200000</v>
+        <v>41400000</v>
       </c>
       <c r="I3" t="n">
-        <v>94.40000000000001</v>
+        <v>92</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -593,103 +617,140 @@
           <t>낙찰</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>20260915</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>방송영상장비;공공방송설비;유지보수</t>
+        </is>
+      </c>
+      <c r="P3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>file:data/procurement/sample_cgi_bids.json</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R26BK00000003-000</t>
+          <t>CGI-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>샘플 물품 공고 C</t>
+          <t>공연장 무대조명 및 음향 설치공사</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>샘플 발주기관</t>
+          <t>샘플 문화재단</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>부산</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>물품</t>
+          <t>공사</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>30000000</v>
+        <v>250000000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>227500000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>91</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>유찰</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+          <t>낙찰</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>20260920</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>음향장비;무대장비;공연장설치</t>
+        </is>
+      </c>
+      <c r="P4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>file:data/procurement/sample_cgi_bids.json</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>R26BK00000004-000</t>
+          <t>CGI-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>샘플 공사 공고 D</t>
+          <t>회의실 영상장비 납품</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>샘플 발주기관</t>
+          <t>샘플 공공기관</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>서울</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>공사</t>
+          <t>물품</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>200000000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>178000000</v>
-      </c>
-      <c r="I5" t="n">
-        <v>89</v>
+        <v>30000000</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>낙찰</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>file:D:\1022\wt-main\data\procurement\sample_bids.json</t>
+          <t>유찰</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>20260925</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>방송영상장비;공공방송설비;기자재납품</t>
+        </is>
+      </c>
+      <c r="P5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>file:data/procurement/sample_cgi_bids.json</t>
         </is>
       </c>
     </row>

</xml_diff>